<commit_message>
pushing to github for the frameworks
</commit_message>
<xml_diff>
--- a/eclipse-workspace/Frameworks/TestData/Data.xlsx
+++ b/eclipse-workspace/Frameworks/TestData/Data.xlsx
@@ -7,9 +7,8 @@
     <workbookView xWindow="240" yWindow="110" windowWidth="14810" windowHeight="8010"/>
   </bookViews>
   <sheets>
-    <sheet name="Login" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Login" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
@@ -362,10 +361,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="14.1796875" customWidth="1"/>
-    <col min="2" max="2" width="17.90625" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -387,13 +382,4 @@
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>